<commit_message>
Đồng bộ hai website theo app bản 224 (Âm nhạc 1 chia tiết đúng SGV KNTT)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RUrX4ZtYx5tevhjTzJSXRj
</commit_message>
<xml_diff>
--- a/assets/docs/lop1/Am nhac - Lop 1.xlsx
+++ b/assets/docs/lop1/Am nhac - Lop 1.xlsx
@@ -542,7 +542,7 @@
       <c r="D4" s="4" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 1: Âm thanh kì diệu — Học hát: Vào rừng hoa (Việt Anh)</t>
+          <t>Chủ đề 1: Âm thanh kì diệu — Thường thức âm nhạc: Âm thanh kì diệu; Học hát: Vào rừng hoa (Việt Anh)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -576,7 +576,7 @@
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 1: Âm thanh kì diệu — Ôn bài hát Vào rừng hoa; Thường thức âm nhạc: Câu chuyện "Âm thanh kì diệu"</t>
+          <t>Chủ đề 1: Âm thanh kì diệu — Ôn bài hát Vào rừng hoa; Đọc nhạc: Bậc thang Đô – Rê – Mi; Vận dụng – Sáng tạo: To – Nhỏ</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -591,7 +591,8 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 1.1 CB1a: HS nghe các đoạn âm thanh GV mở từ học liệu số và nói được đó là tiếng gì.</t>
+          <t>Năng lực số 3.1 CB1a: HS cùng GV tạo bản ghi âm đoạn đọc to – nhỏ của lớp và nghe lại.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -644,7 +645,7 @@
       <c r="D7" s="4" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 1: Âm thanh kì diệu — Vận dụng – Sáng tạo: To – Nhỏ</t>
+          <t>Chủ đề 1: Âm thanh kì diệu — Ôn bài hát Vào rừng hoa; Ôn đọc nhạc: Bậc thang Đô – Rê – Mi; Vận dụng – Sáng tạo: To – Nhỏ</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -659,7 +660,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.1 CB1a: HS cùng GV tạo bản ghi âm đoạn đọc to – nhỏ của lớp và nghe lại.
+          <t>Năng lực số 1.1 CB1a: HS nhìn dòng nhạc Đô – Rê – Mi trên màn hình, nghe tiếng đàn và chỉ ra nốt được đọc to hơn.
 KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
@@ -679,7 +680,7 @@
       <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 2: Việt Nam yêu thương — Học hát: Tổ quốc ta (Mộng Lân)</t>
+          <t>Chủ đề 2: Việt Nam yêu thương — Học hát: Tổ quốc ta (Mộng Lân); Vận dụng – Sáng tạo: Cao – Thấp</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -749,7 +750,7 @@
       <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 2: Việt Nam yêu thương — Nhạc cụ: Gõ đệm trống con cho bài Tổ quốc ta; Nghe nhạc: Quốc ca (Văn Cao)</t>
+          <t>Chủ đề 2: Việt Nam yêu thương — Nghe nhạc: Quốc ca (Văn Cao); Nhạc cụ: Trống con</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -784,7 +785,7 @@
       <c r="D11" s="4" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 2: Việt Nam yêu thương — Vận dụng – Sáng tạo: Cao – Thấp</t>
+          <t>Chủ đề 2: Việt Nam yêu thương — Ôn bài hát Tổ quốc ta; Vận dụng – Sáng tạo: Cao – Thấp</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -799,7 +800,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 1.1 CB1a: HS nghe âm thanh GV mở từ học liệu số và nói được âm nào cao, âm nào thấp.
+          <t>Năng lực số 1.1 CB1a: HS nghe tiếng kèn tu-ba, sáo pic-cô-lô GV mở từ học liệu số và nói được âm nào cao, âm nào thấp.
 QPAN: Chọn bài hát ca ngợi quê hương, đất nước, hoà bình; liên hệ hình ảnh chú bộ đội Quân đội nhân dân, chú công an Công an nhân dân và di tích lịch sử ở địa phương.</t>
         </is>
       </c>
@@ -819,7 +820,7 @@
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 3: Mái trường thân yêu — Học hát: Lớp Một thân yêu (Bùi Anh Tôn)</t>
+          <t>Chủ đề 3: Mái trường thân yêu — Học hát: Lớp Một thân yêu (Bùi Anh Tôn); Vận dụng – Sáng tạo: To – Nhỏ, Cao – Thấp</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -834,7 +835,8 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát Lớp Một thân yêu cùng tên tác giả Bùi Anh Tôn.</t>
+          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát Lớp Một thân yêu cùng tên tác giả Bùi Anh Tôn.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -921,7 +923,7 @@
       <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 3: Mái trường thân yêu — Vận dụng – Sáng tạo: To – Nhỏ, Cao – Thấp</t>
+          <t>Chủ đề 3: Mái trường thân yêu — Ôn bài hát Lớp Một thân yêu; Ôn đọc nhạc: Ban nhạc Đô – Rê – Mi; Vận dụng – Sáng tạo: To – Nhỏ, Cao – Thấp</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1126,7 +1128,7 @@
       <c r="D21" s="4" t="inlineStr"/>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 5: Nhịp điệu mùa xuân — Học hát: Xúc xắc xúc xẻ (Nhạc: Nguyễn Ngọc Thiện, lời: phỏng theo đồng dao)</t>
+          <t>Chủ đề 5: Nhịp điệu mùa xuân — Học hát: Xúc xắc xúc xẻ (Nhạc: Nguyễn Ngọc Thiện, lời: phỏng theo đồng dao); Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1141,7 +1143,8 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát cùng tên tác giả phần nhạc và nguồn lời ca phỏng theo đồng dao.</t>
+          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát cùng tên tác giả phần nhạc và nguồn lời ca phỏng theo đồng dao.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1197,7 @@
       <c r="D23" s="4" t="inlineStr"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 5: Nhịp điệu mùa xuân — Thường thức âm nhạc: Nhạc sĩ Mô-da (Câu chuyện "Thần đồng âm nhạc Mô-da"); Nghe nhạc: Khát vọng mùa xuân</t>
+          <t>Chủ đề 5: Nhịp điệu mùa xuân — Ôn đọc nhạc: Những người bạn của Đô – Rê – Mi; Thường thức âm nhạc: Nhạc sĩ Vôn-gang A-ma-đớt Mô-da (nghe bài hát Khát vọng mùa xuân); Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1209,7 +1212,8 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 1.1 CB1a: HS xem hình, nghe GV giới thiệu và nói được tên nhạc sĩ Mô-da, tên bản nhạc vừa nghe.</t>
+          <t>Năng lực số 1.1 CB1a: HS xem hình, nghe GV giới thiệu và nói được tên nhạc sĩ Mô-da, tên bài hát Khát vọng mùa xuân.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1232,7 @@
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 5: Nhịp điệu mùa xuân — Vận dụng – Sáng tạo: Dài – Ngắn</t>
+          <t>Chủ đề 5: Nhịp điệu mùa xuân — Ôn bài hát Xúc xắc xúc xẻ; Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1263,7 +1267,7 @@
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 6: Về miền dân ca — Học hát: Gà gáy (Dân ca Cống Khao, lời mới: Huy Trân)</t>
+          <t>Chủ đề 6: Về miền dân ca — Học hát: Gà gáy (Dân ca Cống Khao, lời mới: Huy Trân); Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1278,7 +1282,8 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.3 CB1a: HS nói được bài Gà gáy là dân ca Cống Khao và người viết lời mới là Huy Trân.</t>
+          <t>Năng lực số 3.3 CB1a: HS nói được bài Gà gáy là dân ca Cống Khao và người viết lời mới là Huy Trân.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1302,7 @@
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 6: Về miền dân ca — Ôn bài hát Gà gáy; Thường thức âm nhạc: "Câu chuyện về thanh phách"</t>
+          <t>Chủ đề 6: Về miền dân ca — Ôn bài hát Gà gáy; Nhạc cụ: Thanh phách</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1312,7 +1317,7 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 1.1 CB1a: HS xem hình, nghe âm thanh trên màn hình và nói đúng tên nhạc cụ thanh phách.</t>
+          <t>Năng lực số 3.1 CB1a: HS cùng GV ghi âm phần cả lớp hát Gà gáy kết hợp gõ thanh phách và nghe lại để nhận xét tiếng phách đã đều chưa.</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1336,7 @@
       <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 6: Về miền dân ca — Nhạc cụ: Thanh phách; Nghe nhạc: Lí cây bông (Dân ca Nam Bộ)</t>
+          <t>Chủ đề 6: Về miền dân ca — Thường thức âm nhạc: Câu chuyện về thanh phách; Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1346,7 +1351,8 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 4.1 CB1a: HS ngồi đúng khoảng cách với màn hình, nghe loa vừa đủ khi xem, nghe bài Lí cây bông.</t>
+          <t>Năng lực số 1.1 CB1a: HS xem hình, nghe âm thanh trên màn hình và nói đúng tên nhạc cụ thanh phách.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1371,7 @@
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 6: Về miền dân ca — Vận dụng – Sáng tạo: Dài – Ngắn</t>
+          <t>Chủ đề 6: Về miền dân ca — Ôn bài hát Gà gáy; Nghe nhạc: Lí cây bông (Dân ca Nam Bộ)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1380,8 +1386,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 2.1 CB1a: HS nói lời chào buổi sáng để GV ghi lại thành lời nhắn gửi bạn lớp bên.
-KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
+          <t>Năng lực số 4.1 CB1a: HS ngồi đúng khoảng cách với màn hình, nghe loa vừa đủ khi xem, nghe bài Lí cây bông.</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1405,7 @@
       <c r="D29" s="4" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 7: Gia đình — Học hát: Cây gia đình (Nhạc: Quỳnh Hợp, lời thơ: Nguyễn Thị Mai)</t>
+          <t>Chủ đề 7: Gia đình — Học hát: Cây gia đình (Nhạc: Quỳnh Hợp, lời thơ: Nguyễn Thị Mai); Vận dụng – Sáng tạo: Góc âm nhạc</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1415,7 +1420,8 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát cùng tên tác giả nhạc và tác giả lời thơ.</t>
+          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát cùng tên tác giả nhạc và tác giả lời thơ.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1508,7 @@
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 7: Gia đình — Vận dụng – Sáng tạo: Góc âm nhạc</t>
+          <t>Chủ đề 7: Gia đình — Vận dụng – Sáng tạo: Góc âm nhạc; Ôn bài hát Cây gia đình</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1571,7 +1577,7 @@
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 8: Vui đón hè — Ôn bài hát Ngôi sao lấp lánh; Nhạc cụ: Trai-en-gô</t>
+          <t>Chủ đề 8: Vui đón hè — Nhạc cụ: Trai-en-gô (triangle); Ôn bài hát Ngôi sao lấp lánh</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">

</xml_diff>